<commit_message>
Update 700098 - MSCI EM Eastern Europe ex Russia Index .xlsx
</commit_message>
<xml_diff>
--- a/data/700098 - MSCI EM Eastern Europe ex Russia Index .xlsx
+++ b/data/700098 - MSCI EM Eastern Europe ex Russia Index .xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6608" uniqueCount="6607">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6632" uniqueCount="6631">
   <si>
     <t>Index Level:</t>
   </si>
@@ -19832,6 +19832,78 @@
   </si>
   <si>
     <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>2026-03-30</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>2026-04-14</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>2026-04-24</t>
+  </si>
+  <si>
+    <t>2026-04-27</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
   </si>
 </sst>
 </file>
@@ -20217,7 +20289,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:E6592"/>
+  <dimension ref="A3:E6616"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -72990,6 +73062,198 @@
         <v>6859.77894</v>
       </c>
     </row>
+    <row r="6593" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6593" t="s">
+        <v>6607</v>
+      </c>
+      <c r="B6593">
+        <v>6807.2375</v>
+      </c>
+    </row>
+    <row r="6594" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6594" t="s">
+        <v>6608</v>
+      </c>
+      <c r="B6594">
+        <v>6946.915238</v>
+      </c>
+    </row>
+    <row r="6595" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6595" t="s">
+        <v>6609</v>
+      </c>
+      <c r="B6595">
+        <v>7200.058618</v>
+      </c>
+    </row>
+    <row r="6596" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6596" t="s">
+        <v>6610</v>
+      </c>
+      <c r="B6596">
+        <v>7185.875626</v>
+      </c>
+    </row>
+    <row r="6597" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6597" t="s">
+        <v>6611</v>
+      </c>
+      <c r="B6597">
+        <v>7185.875626</v>
+      </c>
+    </row>
+    <row r="6598" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6598" t="s">
+        <v>6612</v>
+      </c>
+      <c r="B6598">
+        <v>7207.856478</v>
+      </c>
+    </row>
+    <row r="6599" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6599" t="s">
+        <v>6613</v>
+      </c>
+      <c r="B6599">
+        <v>7221.659953</v>
+      </c>
+    </row>
+    <row r="6600" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6600" t="s">
+        <v>6614</v>
+      </c>
+      <c r="B6600">
+        <v>7626.706545</v>
+      </c>
+    </row>
+    <row r="6601" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6601" t="s">
+        <v>6615</v>
+      </c>
+      <c r="B6601">
+        <v>7606.741332</v>
+      </c>
+    </row>
+    <row r="6602" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6602" t="s">
+        <v>6616</v>
+      </c>
+      <c r="B6602">
+        <v>7809.86856</v>
+      </c>
+    </row>
+    <row r="6603" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6603" t="s">
+        <v>6617</v>
+      </c>
+      <c r="B6603">
+        <v>7973.227442</v>
+      </c>
+    </row>
+    <row r="6604" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6604" t="s">
+        <v>6618</v>
+      </c>
+      <c r="B6604">
+        <v>8105.799099</v>
+      </c>
+    </row>
+    <row r="6605" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6605" t="s">
+        <v>6619</v>
+      </c>
+      <c r="B6605">
+        <v>8154.870346</v>
+      </c>
+    </row>
+    <row r="6606" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6606" t="s">
+        <v>6620</v>
+      </c>
+      <c r="B6606">
+        <v>8059.629758</v>
+      </c>
+    </row>
+    <row r="6607" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6607" t="s">
+        <v>6621</v>
+      </c>
+      <c r="B6607">
+        <v>8265.81112</v>
+      </c>
+    </row>
+    <row r="6608" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6608" t="s">
+        <v>6622</v>
+      </c>
+      <c r="B6608">
+        <v>8116.739285</v>
+      </c>
+    </row>
+    <row r="6609" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6609" t="s">
+        <v>6623</v>
+      </c>
+      <c r="B6609">
+        <v>8024.305765</v>
+      </c>
+    </row>
+    <row r="6610" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6610" t="s">
+        <v>6624</v>
+      </c>
+      <c r="B6610">
+        <v>7940.073897</v>
+      </c>
+    </row>
+    <row r="6611" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6611" t="s">
+        <v>6625</v>
+      </c>
+      <c r="B6611">
+        <v>7848.155777</v>
+      </c>
+    </row>
+    <row r="6612" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6612" t="s">
+        <v>6626</v>
+      </c>
+      <c r="B6612">
+        <v>7800.014047</v>
+      </c>
+    </row>
+    <row r="6613" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6613" t="s">
+        <v>6627</v>
+      </c>
+      <c r="B6613">
+        <v>7768.533874</v>
+      </c>
+    </row>
+    <row r="6614" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6614" t="s">
+        <v>6628</v>
+      </c>
+      <c r="B6614">
+        <v>7703.841957</v>
+      </c>
+    </row>
+    <row r="6615" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6615" t="s">
+        <v>6629</v>
+      </c>
+      <c r="B6615">
+        <v>7691.488241</v>
+      </c>
+    </row>
+    <row r="6616" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6616" t="s">
+        <v>6630</v>
+      </c>
+      <c r="B6616">
+        <v>7684.876599</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>